<commit_message>
Ajustes estructura de clases (cambio color letra en estilo.css)
</commit_message>
<xml_diff>
--- a/resultados/mi_primera_tabla.xlsx
+++ b/resultados/mi_primera_tabla.xlsx
@@ -401,7 +401,7 @@
         <v>11003.03162536</v>
       </c>
       <c r="C2">
-        <v>9713.20930239591</v>
+        <v>9713.209302395908</v>
       </c>
       <c r="D2">
         <v>275075.790634</v>
@@ -426,10 +426,10 @@
         <v>25054.48163593333</v>
       </c>
       <c r="C3">
-        <v>11800.33981088807</v>
+        <v>11800.33981088806</v>
       </c>
       <c r="D3">
-        <v>751634.4490779999</v>
+        <v>751634.449078</v>
       </c>
       <c r="E3">
         <v>49357.19017</v>

</xml_diff>